<commit_message>
V4 full pipeline latest_pool
</commit_message>
<xml_diff>
--- a/v4_data/runs/latest_pool/25d/result.xlsx
+++ b/v4_data/runs/latest_pool/25d/result.xlsx
@@ -635,7 +635,7 @@
         <v>226555906</v>
       </c>
       <c r="J4" t="n">
-        <v>0.07401786956326846</v>
+        <v>0.0740178695632684</v>
       </c>
       <c r="K4" t="n">
         <v>12.18</v>
@@ -686,7 +686,7 @@
         <v>170775210</v>
       </c>
       <c r="J5" t="n">
-        <v>0.05557057263043718</v>
+        <v>0.0555705726304371</v>
       </c>
       <c r="K5" t="n">
         <v>12.42</v>
@@ -737,7 +737,7 @@
         <v>287239574</v>
       </c>
       <c r="J6" t="n">
-        <v>0.09149756560345165</v>
+        <v>0.0914975656034516</v>
       </c>
       <c r="K6" t="n">
         <v>12.73</v>
@@ -788,7 +788,7 @@
         <v>248827502</v>
       </c>
       <c r="J7" t="n">
-        <v>0.07997879814014834</v>
+        <v>0.0799787981401483</v>
       </c>
       <c r="K7" t="n">
         <v>12.69</v>
@@ -839,7 +839,7 @@
         <v>358573912</v>
       </c>
       <c r="J8" t="n">
-        <v>0.1140199455875327</v>
+        <v>0.1140199455875326</v>
       </c>
       <c r="K8" t="n">
         <v>12.97</v>
@@ -992,7 +992,7 @@
         <v>372583228</v>
       </c>
       <c r="J11" t="n">
-        <v>0.1113355333670319</v>
+        <v>0.1113355333670318</v>
       </c>
       <c r="K11" t="n">
         <v>13.52</v>
@@ -1043,7 +1043,7 @@
         <v>248782419</v>
       </c>
       <c r="J12" t="n">
-        <v>0.07515817665519671</v>
+        <v>0.0751581766551967</v>
       </c>
       <c r="K12" t="n">
         <v>13.4</v>
@@ -1145,7 +1145,7 @@
         <v>223186371</v>
       </c>
       <c r="J14" t="n">
-        <v>0.06883435499854522</v>
+        <v>0.06883435499854521</v>
       </c>
       <c r="K14" t="n">
         <v>13.4</v>
@@ -1247,7 +1247,7 @@
         <v>340236879</v>
       </c>
       <c r="J16" t="n">
-        <v>0.09027037618771998</v>
+        <v>0.09027037618771989</v>
       </c>
       <c r="K16" t="n">
         <v>14.5</v>
@@ -1808,7 +1808,7 @@
         <v>551014807</v>
       </c>
       <c r="J27" t="n">
-        <v>0.01845488513634565</v>
+        <v>0.0184548851363456</v>
       </c>
       <c r="K27" t="n">
         <v>21.26</v>
@@ -1859,7 +1859,7 @@
         <v>314817831</v>
       </c>
       <c r="J28" t="n">
-        <v>0.01042250987800605</v>
+        <v>0.010422509878006</v>
       </c>
       <c r="K28" t="n">
         <v>22.61</v>
@@ -1910,7 +1910,7 @@
         <v>301519512</v>
       </c>
       <c r="J29" t="n">
-        <v>0.01012785258297788</v>
+        <v>0.0101278525829778</v>
       </c>
       <c r="K29" t="n">
         <v>21.9</v>
@@ -1961,7 +1961,7 @@
         <v>678835270</v>
       </c>
       <c r="J30" t="n">
-        <v>0.02337843553901912</v>
+        <v>0.0233784355390191</v>
       </c>
       <c r="K30" t="n">
         <v>22.2</v>
@@ -2012,7 +2012,7 @@
         <v>350258216</v>
       </c>
       <c r="J31" t="n">
-        <v>0.01238894620735823</v>
+        <v>0.0123889462073582</v>
       </c>
       <c r="K31" t="n">
         <v>21.22</v>
@@ -2063,7 +2063,7 @@
         <v>303971260</v>
       </c>
       <c r="J32" t="n">
-        <v>0.01042918798466196</v>
+        <v>0.0104291879846619</v>
       </c>
       <c r="K32" t="n">
         <v>21.4</v>
@@ -2114,7 +2114,7 @@
         <v>542397305</v>
       </c>
       <c r="J33" t="n">
-        <v>0.01777214115100532</v>
+        <v>0.0177721411510053</v>
       </c>
       <c r="K33" t="n">
         <v>21.93</v>
@@ -2165,7 +2165,7 @@
         <v>336402761</v>
       </c>
       <c r="J34" t="n">
-        <v>0.01088417648408654</v>
+        <v>0.0108841764840865</v>
       </c>
       <c r="K34" t="n">
         <v>22.91</v>
@@ -2216,7 +2216,7 @@
         <v>430055151</v>
       </c>
       <c r="J35" t="n">
-        <v>0.01356345747014125</v>
+        <v>0.0135634574701412</v>
       </c>
       <c r="K35" t="n">
         <v>22.8</v>
@@ -2267,7 +2267,7 @@
         <v>356332289</v>
       </c>
       <c r="J36" t="n">
-        <v>0.01099282391304242</v>
+        <v>0.0109928239130424</v>
       </c>
       <c r="K36" t="n">
         <v>23.81</v>
@@ -2369,7 +2369,7 @@
         <v>269444127</v>
       </c>
       <c r="J38" t="n">
-        <v>0.008721869646802966</v>
+        <v>0.0087218696468029</v>
       </c>
       <c r="K38" t="n">
         <v>23.41</v>
@@ -2420,7 +2420,7 @@
         <v>169081167</v>
       </c>
       <c r="J39" t="n">
-        <v>0.00551535810285973</v>
+        <v>0.0055153581028597</v>
       </c>
       <c r="K39" t="n">
         <v>22.92</v>
@@ -2471,7 +2471,7 @@
         <v>174316168</v>
       </c>
       <c r="J40" t="n">
-        <v>0.005678717560307807</v>
+        <v>0.0056787175603078</v>
       </c>
       <c r="K40" t="n">
         <v>23.1</v>
@@ -2522,7 +2522,7 @@
         <v>158979880</v>
       </c>
       <c r="J41" t="n">
-        <v>0.005215521548551211</v>
+        <v>0.0052155215485512</v>
       </c>
       <c r="K41" t="n">
         <v>22.76</v>
@@ -2573,7 +2573,7 @@
         <v>199460425</v>
       </c>
       <c r="J42" t="n">
-        <v>0.006478980570979595</v>
+        <v>0.0064789805709795</v>
       </c>
       <c r="K42" t="n">
         <v>22.76</v>
@@ -2624,7 +2624,7 @@
         <v>280003976</v>
       </c>
       <c r="J43" t="n">
-        <v>0.009064582478075133</v>
+        <v>0.0090645824780751</v>
       </c>
       <c r="K43" t="n">
         <v>22.95</v>
@@ -2675,7 +2675,7 @@
         <v>224449129</v>
       </c>
       <c r="J44" t="n">
-        <v>0.00730665586788995</v>
+        <v>0.0073066558678899</v>
       </c>
       <c r="K44" t="n">
         <v>22.72</v>
@@ -2726,7 +2726,7 @@
         <v>305117293</v>
       </c>
       <c r="J45" t="n">
-        <v>0.009611964371862739</v>
+        <v>0.009611964371862699</v>
       </c>
       <c r="K45" t="n">
         <v>23</v>
@@ -2777,7 +2777,7 @@
         <v>159254942</v>
       </c>
       <c r="J46" t="n">
-        <v>0.00509852052368022</v>
+        <v>0.0050985205236802</v>
       </c>
       <c r="K46" t="n">
         <v>23.25</v>
@@ -2828,7 +2828,7 @@
         <v>224342247</v>
       </c>
       <c r="J47" t="n">
-        <v>0.006978366554475493</v>
+        <v>0.0069783665544754</v>
       </c>
       <c r="K47" t="n">
         <v>23.4</v>
@@ -2879,7 +2879,7 @@
         <v>109972224</v>
       </c>
       <c r="J48" t="n">
-        <v>0.003439851000290454</v>
+        <v>0.0034398510002904</v>
       </c>
       <c r="K48" t="n">
         <v>23.86</v>
@@ -2930,7 +2930,7 @@
         <v>144386613</v>
       </c>
       <c r="J49" t="n">
-        <v>0.004466803682980889</v>
+        <v>0.0044668036829808</v>
       </c>
       <c r="K49" t="n">
         <v>24.06</v>
@@ -3032,7 +3032,7 @@
         <v>303128374</v>
       </c>
       <c r="J51" t="n">
-        <v>0.009384530866089339</v>
+        <v>0.0093845308660893</v>
       </c>
       <c r="K51" t="n">
         <v>23.46</v>
@@ -3083,7 +3083,7 @@
         <v>102254152</v>
       </c>
       <c r="J52" t="n">
-        <v>0.01753733994718489</v>
+        <v>0.0175373399471848</v>
       </c>
       <c r="K52" t="n">
         <v>5.01</v>
@@ -3134,7 +3134,7 @@
         <v>166132703</v>
       </c>
       <c r="J53" t="n">
-        <v>0.02783904780984943</v>
+        <v>0.0278390478098494</v>
       </c>
       <c r="K53" t="n">
         <v>5.07</v>
@@ -3185,7 +3185,7 @@
         <v>140629024</v>
       </c>
       <c r="J54" t="n">
-        <v>0.02342215497194439</v>
+        <v>0.0234221549719443</v>
       </c>
       <c r="K54" t="n">
         <v>5.15</v>
@@ -3236,7 +3236,7 @@
         <v>115096284</v>
       </c>
       <c r="J55" t="n">
-        <v>0.01880352479724743</v>
+        <v>0.0188035247972474</v>
       </c>
       <c r="K55" t="n">
         <v>5.27</v>
@@ -3287,7 +3287,7 @@
         <v>109185278</v>
       </c>
       <c r="J56" t="n">
-        <v>0.01795755286176362</v>
+        <v>0.0179575528617636</v>
       </c>
       <c r="K56" t="n">
         <v>5.34</v>
@@ -3338,7 +3338,7 @@
         <v>142175559</v>
       </c>
       <c r="J57" t="n">
-        <v>0.02358295903769857</v>
+        <v>0.0235829590376985</v>
       </c>
       <c r="K57" t="n">
         <v>5.28</v>
@@ -3389,7 +3389,7 @@
         <v>181721476</v>
       </c>
       <c r="J58" t="n">
-        <v>0.0306089825372349</v>
+        <v>0.0306089825372348</v>
       </c>
       <c r="K58" t="n">
         <v>5.22</v>
@@ -3440,7 +3440,7 @@
         <v>119283839</v>
       </c>
       <c r="J59" t="n">
-        <v>0.02036619303958408</v>
+        <v>0.020366193039584</v>
       </c>
       <c r="K59" t="n">
         <v>5.16</v>
@@ -3491,7 +3491,7 @@
         <v>178080803</v>
       </c>
       <c r="J60" t="n">
-        <v>0.02938558516327045</v>
+        <v>0.0293855851632704</v>
       </c>
       <c r="K60" t="n">
         <v>5.2</v>
@@ -3542,7 +3542,7 @@
         <v>120278990</v>
       </c>
       <c r="J61" t="n">
-        <v>0.01991397901330254</v>
+        <v>0.0199139790133025</v>
       </c>
       <c r="K61" t="n">
         <v>5.31</v>
@@ -3593,7 +3593,7 @@
         <v>104097943</v>
       </c>
       <c r="J62" t="n">
-        <v>0.01725257871070722</v>
+        <v>0.0172525787107072</v>
       </c>
       <c r="K62" t="n">
         <v>5.19</v>
@@ -3644,7 +3644,7 @@
         <v>125223561</v>
       </c>
       <c r="J63" t="n">
-        <v>0.02079142638379678</v>
+        <v>0.0207914263837967</v>
       </c>
       <c r="K63" t="n">
         <v>5.26</v>
@@ -3746,7 +3746,7 @@
         <v>480537096</v>
       </c>
       <c r="J65" t="n">
-        <v>0.07658850653337537</v>
+        <v>0.0765885065333753</v>
       </c>
       <c r="K65" t="n">
         <v>5.4</v>
@@ -4001,7 +4001,7 @@
         <v>386339879</v>
       </c>
       <c r="J70" t="n">
-        <v>0.06351162976746608</v>
+        <v>0.06351162976746599</v>
       </c>
       <c r="K70" t="n">
         <v>5.4</v>
@@ -4052,7 +4052,7 @@
         <v>414588063</v>
       </c>
       <c r="J71" t="n">
-        <v>0.06661426223235131</v>
+        <v>0.0666142622323513</v>
       </c>
       <c r="K71" t="n">
         <v>5.25</v>
@@ -4103,7 +4103,7 @@
         <v>403201143</v>
       </c>
       <c r="J72" t="n">
-        <v>0.06315764082059445</v>
+        <v>0.0631576408205944</v>
       </c>
       <c r="K72" t="n">
         <v>5.39</v>
@@ -4154,7 +4154,7 @@
         <v>450240950</v>
       </c>
       <c r="J73" t="n">
-        <v>0.06895346790464923</v>
+        <v>0.06895346790464919</v>
       </c>
       <c r="K73" t="n">
         <v>5.52</v>
@@ -4205,7 +4205,7 @@
         <v>395176509</v>
       </c>
       <c r="J74" t="n">
-        <v>0.05902490621152327</v>
+        <v>0.0590249062115232</v>
       </c>
       <c r="K74" t="n">
         <v>5.85</v>
@@ -4256,7 +4256,7 @@
         <v>351718999</v>
       </c>
       <c r="J75" t="n">
-        <v>0.05304068442090487</v>
+        <v>0.0530406844209048</v>
       </c>
       <c r="K75" t="n">
         <v>5.88</v>
@@ -4358,7 +4358,7 @@
         <v>48956785</v>
       </c>
       <c r="J77" t="n">
-        <v>0.007904718108655631</v>
+        <v>0.0079047181086556</v>
       </c>
       <c r="K77" t="n">
         <v>3.8</v>
@@ -4409,7 +4409,7 @@
         <v>51499663</v>
       </c>
       <c r="J78" t="n">
-        <v>0.008253002304797384</v>
+        <v>0.008253002304797301</v>
       </c>
       <c r="K78" t="n">
         <v>3.85</v>
@@ -4460,7 +4460,7 @@
         <v>48521583</v>
       </c>
       <c r="J79" t="n">
-        <v>0.007811177500995373</v>
+        <v>0.0078111775009953</v>
       </c>
       <c r="K79" t="n">
         <v>3.86</v>
@@ -4511,7 +4511,7 @@
         <v>120273053</v>
       </c>
       <c r="J80" t="n">
-        <v>0.01891437767734037</v>
+        <v>0.0189143776773403</v>
       </c>
       <c r="K80" t="n">
         <v>3.88</v>
@@ -4562,7 +4562,7 @@
         <v>98551722</v>
       </c>
       <c r="J81" t="n">
-        <v>0.01568473549423195</v>
+        <v>0.0156847354942319</v>
       </c>
       <c r="K81" t="n">
         <v>3.96</v>
@@ -4613,7 +4613,7 @@
         <v>76896290</v>
       </c>
       <c r="J82" t="n">
-        <v>0.01220378275886442</v>
+        <v>0.0122037827588644</v>
       </c>
       <c r="K82" t="n">
         <v>3.89</v>
@@ -4664,7 +4664,7 @@
         <v>58290689</v>
       </c>
       <c r="J83" t="n">
-        <v>0.00927591477247899</v>
+        <v>0.0092759147724789</v>
       </c>
       <c r="K83" t="n">
         <v>3.92</v>
@@ -4715,7 +4715,7 @@
         <v>43949443</v>
       </c>
       <c r="J84" t="n">
-        <v>0.006975407131288968</v>
+        <v>0.0069754071312889</v>
       </c>
       <c r="K84" t="n">
         <v>3.94</v>
@@ -4766,7 +4766,7 @@
         <v>132807140</v>
       </c>
       <c r="J85" t="n">
-        <v>0.02061867390622562</v>
+        <v>0.0206186739062256</v>
       </c>
       <c r="K85" t="n">
         <v>3.92</v>
@@ -4817,7 +4817,7 @@
         <v>96406563</v>
       </c>
       <c r="J86" t="n">
-        <v>0.01497864207274804</v>
+        <v>0.014978642072748</v>
       </c>
       <c r="K86" t="n">
         <v>4.03</v>
@@ -4868,7 +4868,7 @@
         <v>55331737</v>
       </c>
       <c r="J87" t="n">
-        <v>0.008595586517707088</v>
+        <v>0.008595586517706999</v>
       </c>
       <c r="K87" t="n">
         <v>3.99</v>
@@ -4919,7 +4919,7 @@
         <v>65346684</v>
       </c>
       <c r="J88" t="n">
-        <v>0.01021759797502998</v>
+        <v>0.0102175979750299</v>
       </c>
       <c r="K88" t="n">
         <v>4.02</v>
@@ -4970,7 +4970,7 @@
         <v>64618943</v>
       </c>
       <c r="J89" t="n">
-        <v>0.01018251279213844</v>
+        <v>0.0101825127921384</v>
       </c>
       <c r="K89" t="n">
         <v>3.96</v>
@@ -5021,7 +5021,7 @@
         <v>51680997</v>
       </c>
       <c r="J90" t="n">
-        <v>0.008120716721197086</v>
+        <v>0.008120716721197</v>
       </c>
       <c r="K90" t="n">
         <v>3.93</v>
@@ -5072,7 +5072,7 @@
         <v>46789375</v>
       </c>
       <c r="J91" t="n">
-        <v>0.007311617303004035</v>
+        <v>0.007311617303004</v>
       </c>
       <c r="K91" t="n">
         <v>3.97</v>
@@ -5123,7 +5123,7 @@
         <v>53140094</v>
       </c>
       <c r="J92" t="n">
-        <v>0.008352355342225384</v>
+        <v>0.008352355342225301</v>
       </c>
       <c r="K92" t="n">
         <v>3.97</v>
@@ -5174,7 +5174,7 @@
         <v>36978724</v>
       </c>
       <c r="J93" t="n">
-        <v>0.00582495854832412</v>
+        <v>0.0058249585483241</v>
       </c>
       <c r="K93" t="n">
         <v>3.93</v>
@@ -5225,7 +5225,7 @@
         <v>172671281</v>
       </c>
       <c r="J94" t="n">
-        <v>0.02652454923013641</v>
+        <v>0.0265245492301364</v>
       </c>
       <c r="K94" t="n">
         <v>4.1</v>
@@ -5276,7 +5276,7 @@
         <v>109158107</v>
       </c>
       <c r="J95" t="n">
-        <v>0.01676797646019123</v>
+        <v>0.0167679764601912</v>
       </c>
       <c r="K95" t="n">
         <v>4.02</v>
@@ -5327,7 +5327,7 @@
         <v>182545656</v>
       </c>
       <c r="J96" t="n">
-        <v>0.02750565581535108</v>
+        <v>0.027505655815351</v>
       </c>
       <c r="K96" t="n">
         <v>4.05</v>
@@ -5378,7 +5378,7 @@
         <v>272727382</v>
       </c>
       <c r="J97" t="n">
-        <v>0.04011489220435863</v>
+        <v>0.0401148922043586</v>
       </c>
       <c r="K97" t="n">
         <v>4.16</v>
@@ -5429,7 +5429,7 @@
         <v>161769736</v>
       </c>
       <c r="J98" t="n">
-        <v>0.02354123329787341</v>
+        <v>0.0235412332978734</v>
       </c>
       <c r="K98" t="n">
         <v>4.29</v>
@@ -5480,7 +5480,7 @@
         <v>248731055</v>
       </c>
       <c r="J99" t="n">
-        <v>0.03551433664814662</v>
+        <v>0.0355143366481466</v>
       </c>
       <c r="K99" t="n">
         <v>4.25</v>
@@ -5531,7 +5531,7 @@
         <v>145447912</v>
       </c>
       <c r="J100" t="n">
-        <v>0.02083509310608567</v>
+        <v>0.0208350931060856</v>
       </c>
       <c r="K100" t="n">
         <v>4.4</v>
@@ -5582,7 +5582,7 @@
         <v>155547202</v>
       </c>
       <c r="J101" t="n">
-        <v>0.02199025512477603</v>
+        <v>0.021990255124776</v>
       </c>
       <c r="K101" t="n">
         <v>4.34</v>
@@ -5633,7 +5633,7 @@
         <v>376584591</v>
       </c>
       <c r="J102" t="n">
-        <v>0.02193926245154992</v>
+        <v>0.0219392624515499</v>
       </c>
       <c r="K102" t="n">
         <v>9.65</v>
@@ -5684,7 +5684,7 @@
         <v>298488541</v>
       </c>
       <c r="J103" t="n">
-        <v>0.01753103288051672</v>
+        <v>0.0175310328805167</v>
       </c>
       <c r="K103" t="n">
         <v>9.949999999999999</v>
@@ -5735,7 +5735,7 @@
         <v>265283500</v>
       </c>
       <c r="J104" t="n">
-        <v>0.01540541688124092</v>
+        <v>0.0154054168812409</v>
       </c>
       <c r="K104" t="n">
         <v>10</v>
@@ -5786,7 +5786,7 @@
         <v>167445936</v>
       </c>
       <c r="J105" t="n">
-        <v>0.009739176808758616</v>
+        <v>0.0097391768087586</v>
       </c>
       <c r="K105" t="n">
         <v>9.84</v>
@@ -5837,7 +5837,7 @@
         <v>233671365</v>
       </c>
       <c r="J106" t="n">
-        <v>0.01335587521639353</v>
+        <v>0.0133558752163935</v>
       </c>
       <c r="K106" t="n">
         <v>9.960000000000001</v>
@@ -5888,7 +5888,7 @@
         <v>279004852</v>
       </c>
       <c r="J107" t="n">
-        <v>0.01553995573439236</v>
+        <v>0.0155399557343923</v>
       </c>
       <c r="K107" t="n">
         <v>10.24</v>
@@ -5939,7 +5939,7 @@
         <v>295178900</v>
       </c>
       <c r="J108" t="n">
-        <v>0.01650252789480048</v>
+        <v>0.0165025278948004</v>
       </c>
       <c r="K108" t="n">
         <v>10.53</v>
@@ -6041,7 +6041,7 @@
         <v>261045144</v>
       </c>
       <c r="J110" t="n">
-        <v>0.01447437532117515</v>
+        <v>0.0144743753211751</v>
       </c>
       <c r="K110" t="n">
         <v>10.56</v>
@@ -6092,7 +6092,7 @@
         <v>217048168</v>
       </c>
       <c r="J111" t="n">
-        <v>0.01221077035407143</v>
+        <v>0.0122107703540714</v>
       </c>
       <c r="K111" t="n">
         <v>10.36</v>
@@ -6143,7 +6143,7 @@
         <v>155775404</v>
       </c>
       <c r="J112" t="n">
-        <v>0.008815156960956954</v>
+        <v>0.0088151569609569</v>
       </c>
       <c r="K112" t="n">
         <v>10.18</v>
@@ -6194,7 +6194,7 @@
         <v>266420998</v>
       </c>
       <c r="J113" t="n">
-        <v>0.01531626751463312</v>
+        <v>0.0153162675146331</v>
       </c>
       <c r="K113" t="n">
         <v>10.23</v>
@@ -6245,7 +6245,7 @@
         <v>636052606</v>
       </c>
       <c r="J114" t="n">
-        <v>0.03424924558519227</v>
+        <v>0.0342492455851922</v>
       </c>
       <c r="K114" t="n">
         <v>10.1</v>
@@ -6296,7 +6296,7 @@
         <v>1535040772</v>
       </c>
       <c r="J115" t="n">
-        <v>0.07735375195427029</v>
+        <v>0.0773537519542702</v>
       </c>
       <c r="K115" t="n">
         <v>11.29</v>
@@ -6347,7 +6347,7 @@
         <v>1072241949</v>
       </c>
       <c r="J116" t="n">
-        <v>0.05277038443868282</v>
+        <v>0.0527703844386828</v>
       </c>
       <c r="K116" t="n">
         <v>11.75</v>
@@ -6398,7 +6398,7 @@
         <v>2615213529</v>
       </c>
       <c r="J117" t="n">
-        <v>0.1179636455018439</v>
+        <v>0.1179636455018438</v>
       </c>
       <c r="K117" t="n">
         <v>11.89</v>
@@ -6449,7 +6449,7 @@
         <v>1905394843</v>
       </c>
       <c r="J118" t="n">
-        <v>0.08635243199211207</v>
+        <v>0.086352431992112</v>
       </c>
       <c r="K118" t="n">
         <v>12.83</v>
@@ -6500,7 +6500,7 @@
         <v>1401406868</v>
       </c>
       <c r="J119" t="n">
-        <v>0.06138113541032933</v>
+        <v>0.0613811354103293</v>
       </c>
       <c r="K119" t="n">
         <v>12.86</v>
@@ -6551,7 +6551,7 @@
         <v>1271106722</v>
       </c>
       <c r="J120" t="n">
-        <v>0.05543506870786812</v>
+        <v>0.0554350687078681</v>
       </c>
       <c r="K120" t="n">
         <v>13.1</v>
@@ -6602,7 +6602,7 @@
         <v>978161080</v>
       </c>
       <c r="J121" t="n">
-        <v>0.04236031015427182</v>
+        <v>0.0423603101542718</v>
       </c>
       <c r="K121" t="n">
         <v>13.12</v>
@@ -6653,7 +6653,7 @@
         <v>777599360</v>
       </c>
       <c r="J122" t="n">
-        <v>0.03369374241287517</v>
+        <v>0.0336937424128751</v>
       </c>
       <c r="K122" t="n">
         <v>13.46</v>
@@ -6704,7 +6704,7 @@
         <v>884540012</v>
       </c>
       <c r="J123" t="n">
-        <v>0.03850909477157433</v>
+        <v>0.0385090947715743</v>
       </c>
       <c r="K123" t="n">
         <v>13.17</v>
@@ -6755,7 +6755,7 @@
         <v>597568658</v>
       </c>
       <c r="J124" t="n">
-        <v>0.02644063181357697</v>
+        <v>0.0264406318135769</v>
       </c>
       <c r="K124" t="n">
         <v>13.3</v>
@@ -6806,7 +6806,7 @@
         <v>753175705</v>
       </c>
       <c r="J125" t="n">
-        <v>0.03325841129324163</v>
+        <v>0.0332584112932416</v>
       </c>
       <c r="K125" t="n">
         <v>12.63</v>
@@ -6857,7 +6857,7 @@
         <v>556790078</v>
       </c>
       <c r="J126" t="n">
-        <v>0.02385972447387665</v>
+        <v>0.0238597244738766</v>
       </c>
       <c r="K126" t="n">
         <v>13.6</v>
@@ -6952,12 +6952,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>sina</t>
+          <t>cache</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>sina</t>
+          <t>cache</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -6986,12 +6986,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>sina</t>
+          <t>cache</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>sina</t>
+          <t>cache</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -7020,12 +7020,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>sina</t>
+          <t>cache</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>sina</t>
+          <t>cache</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -7054,12 +7054,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>sina</t>
+          <t>cache</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>sina</t>
+          <t>cache</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -7088,12 +7088,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>sina</t>
+          <t>cache</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>sina</t>
+          <t>cache</t>
         </is>
       </c>
       <c r="G6" t="n">

</xml_diff>